<commit_message>
Attribution rerun (13a-d, 14, 15) for seed 7
Replaces the attribution outputs that were stale copies from the initial commit.
Run on 24-09-2026 with tools/run_pipeline.py --only 13a 13b 13c 13d 14 15;
log in thesis-ews-final/outputs/run_logs/seed_attribution_2409.log.
Bank-level SHAP values stay out of the repository (gitignored, licensed data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/appendix_direction.xlsx
+++ b/outputs/tables/appendix_direction.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.927</v>
+        <v>1.033</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.87</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.654</v>
+        <v>0.827</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -541,12 +541,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.571</v>
+        <v>0.662</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.55</v>
+        <v>-0.52</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.328</v>
+        <v>0.415</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -618,33 +618,33 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Inflation (CPI)</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PCPIPCH</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -653,41 +653,41 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.277</v>
+        <v>0.333</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.35</v>
+        <v>-0.44</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Inflation (CPI)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>PCPIPCH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -696,24 +696,24 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.256</v>
+        <v>0.291</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.42</v>
+        <v>0.38</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.119</v>
+        <v>0.208</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -756,7 +756,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.101</v>
+        <v>0.154</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.51</v>
+        <v>0.76</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -799,7 +799,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.091</v>
+        <v>0.135</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.43</v>
+        <v>0.17</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -854,12 +854,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.055</v>
+        <v>0.061</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.48</v>
+        <v>-0.57</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -885,24 +885,24 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -911,15 +911,15 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.043</v>
+        <v>0.059</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.45</v>
+        <v>0.73</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -928,24 +928,24 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -954,41 +954,41 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.028</v>
+        <v>0.04</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.72</v>
+        <v>-0.52</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Log loans</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>l_loans</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -997,41 +997,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.023</v>
+        <v>0.037</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-0.35</v>
+        <v>-0.38</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1040,41 +1040,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.018</v>
+        <v>0.025</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.33</v>
+        <v>-0.48</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>5/6</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.017</v>
+        <v>0.022</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1091,16 +1091,16 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.15</v>
+        <v>-0.45</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1112,12 +1112,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1126,41 +1126,41 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>0.59</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.016</v>
+        <v>0.019</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.02</v>
+        <v>-0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1220,16 +1220,16 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Log loans</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>l_loans</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1263,11 +1263,11 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.21</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1284,12 +1284,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1306,16 +1306,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>-0.36</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1327,12 +1327,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.02</v>
+        <v>0.22</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1370,12 +1370,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1392,7 +1392,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>-0.05</v>
+        <v>-0.35</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1413,12 +1413,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1435,16 +1435,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-0.08</v>
+        <v>0.17</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>3/6</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1/6</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1456,12 +1456,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1478,16 +1478,16 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.14</v>
+        <v>0.16</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.792</v>
+        <v>0.718</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.88</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.556</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.492</v>
+        <v>0.463</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.53</v>
+        <v>-0.54</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1689,12 +1689,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Credit growth</t>
+          <t>Change in net foreign assets (% GDP)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>credit_g</t>
+          <t>nfa_gdp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.293</v>
+        <v>0.309</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1732,12 +1732,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Credit-to-GDP gap</t>
+          <t>Credit growth</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>credit_gap</t>
+          <t>credit_g</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.272</v>
+        <v>0.276</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-0.64</v>
+        <v>-0.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1775,12 +1775,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nominal GDP (log)</t>
+          <t>Private credit (% GDP)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NGDPD</t>
+          <t>FS.AST.PRVT.GD.ZS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.19</v>
+        <v>0.268</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1797,16 +1797,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.84</v>
+        <v>0.63</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1818,12 +1818,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Credit-to-GDP gap</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>credit_gap</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.186</v>
+        <v>0.25</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.49</v>
+        <v>-0.57</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1861,12 +1861,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private credit (% GDP)</t>
+          <t>Nominal GDP (log)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FS.AST.PRVT.GD.ZS</t>
+          <t>NGDPD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.179</v>
+        <v>0.249</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1892,12 +1892,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.157</v>
+        <v>0.207</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.47</v>
+        <v>0.59</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1947,12 +1947,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Net foreign assets growth</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nfa_g</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.147</v>
+        <v>0.205</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1969,11 +1969,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.32</v>
+        <v>-0.45</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.108</v>
+        <v>0.133</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2033,12 +2033,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Current account (% GDP)</t>
+          <t>Real effective exchange rate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BCA_NGDPD</t>
+          <t>BIS_REER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2047,15 +2047,15 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.103</v>
+        <v>0.124</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-0.42</v>
+        <v>0.54</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2076,12 +2076,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Real effective exchange rate</t>
+          <t>Current account (% GDP)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BIS_REER</t>
+          <t>BCA_NGDPD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2090,41 +2090,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.09</v>
+        <v>0.097</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.64</v>
+        <v>-0.15</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2133,41 +2133,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.057</v>
+        <v>0.031</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.51</v>
+        <v>-0.64</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2176,41 +2176,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.044</v>
+        <v>0.026</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>-0.47</v>
+        <v>0.8</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2219,15 +2219,15 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.035</v>
+        <v>0.017</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-0.24</v>
+        <v>-0.61</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2236,24 +2236,24 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2270,16 +2270,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-0.29</v>
+        <v>0.09</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2291,12 +2291,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Loans-to-deposits</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>r_loans_dep</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2305,41 +2305,41 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.027</v>
+        <v>0.014</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-0.06</v>
+        <v>-0.49</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Loans-to-deposits</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>r_loans_dep</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2348,41 +2348,41 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.026</v>
+        <v>0.014</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-0.32</v>
+        <v>-0.01</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.017</v>
+        <v>0.013</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2399,16 +2399,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>-0.09</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2420,12 +2420,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Log off-balance-sheet items</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>l_obsi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2434,41 +2434,41 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>-0.36</v>
+        <v>0.55</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Impairment charges</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>cr_impchg</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2485,16 +2485,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.06</v>
+        <v>0.24</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2506,12 +2506,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Impairment charges</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cr_impchg</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2520,29 +2520,29 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17</v>
+        <v>-0.41</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.33</v>
+        <v>-0.5</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2592,12 +2592,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Log off-balance-sheet items</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>l_obsi</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2606,19 +2606,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.014</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.41</v>
+        <v>0.17</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.012</v>
+        <v>0.007</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.12</v>
+        <v>0.23</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2678,12 +2678,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2692,19 +2692,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-0.02</v>
+        <v>0.31</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2714,19 +2714,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2743,16 +2743,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>-0.05</v>
+        <v>0.53</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2764,12 +2764,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.004</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2786,16 +2786,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.05</v>
+        <v>0.26</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2807,12 +2807,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.26</v>
+        <v>-0.35</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">

</xml_diff>

<commit_message>
Attribution rerun (13a-d, 14, 15) for seed 13
Replaces the attribution outputs that were stale copies from the initial commit.
Run on 24-09-2026 with tools/run_pipeline.py --only 13a 13b 13c 13d 14 15;
log in thesis-ews-final/outputs/run_logs/seed_attribution_2409.log.
Bank-level SHAP values stay out of the repository (gitignored, licensed data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/appendix_direction.xlsx
+++ b/outputs/tables/appendix_direction.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.927</v>
+        <v>0.96</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.88</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.654</v>
+        <v>0.733</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -541,12 +541,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.571</v>
+        <v>0.569</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -575,11 +575,11 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.55</v>
+        <v>-0.46</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.328</v>
+        <v>0.374</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -618,21 +618,21 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.277</v>
+        <v>0.271</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.256</v>
+        <v>0.244</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.42</v>
+        <v>-0.48</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.119</v>
+        <v>0.17</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -747,16 +747,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.05</v>
+        <v>-0.03</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.101</v>
+        <v>0.123</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.51</v>
+        <v>0.65</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -799,7 +799,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.091</v>
+        <v>0.095</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -833,16 +833,16 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.43</v>
+        <v>0.35</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/5</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -854,12 +854,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.48</v>
+        <v>-0.66</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -897,12 +897,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -911,15 +911,15 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.45</v>
+        <v>0.74</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -928,24 +928,24 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Log loans</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>l_loans</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -954,41 +954,41 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.028</v>
+        <v>0.038</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.72</v>
+        <v>0.19</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.023</v>
+        <v>0.036</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-0.35</v>
+        <v>-0.4</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1026,12 +1026,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1040,41 +1040,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.33</v>
+        <v>-0.37</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1091,16 +1091,16 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.15</v>
+        <v>0.4</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1112,12 +1112,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.017</v>
+        <v>0.015</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1134,16 +1134,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>-0.17</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>3/6</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2/6</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1155,12 +1155,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1220,11 +1220,11 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.24</v>
+        <v>0.63</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Log loans</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>l_loans</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.016</v>
+        <v>0.011</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1263,16 +1263,16 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.21</v>
+        <v>-0.36</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1284,12 +1284,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1298,41 +1298,41 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>-0.59</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1341,15 +1341,15 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.02</v>
+        <v>-0.62</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1358,24 +1358,24 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1392,16 +1392,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>-0.05</v>
+        <v>0.18</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1413,12 +1413,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.006</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1435,16 +1435,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1456,12 +1456,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1478,7 +1478,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.14</v>
+        <v>0.12</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.792</v>
+        <v>0.705</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.87</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.556</v>
+        <v>0.596</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.492</v>
+        <v>0.496</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.53</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1689,12 +1689,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Credit growth</t>
+          <t>Change in net foreign assets (% GDP)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>credit_g</t>
+          <t>nfa_gdp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.293</v>
+        <v>0.317</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-0.7</v>
+        <v>-0.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1732,12 +1732,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Credit-to-GDP gap</t>
+          <t>Credit growth</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>credit_gap</t>
+          <t>credit_g</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.272</v>
+        <v>0.292</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-0.64</v>
+        <v>-0.62</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1775,12 +1775,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nominal GDP (log)</t>
+          <t>Private credit (% GDP)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NGDPD</t>
+          <t>FS.AST.PRVT.GD.ZS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.19</v>
+        <v>0.284</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1797,16 +1797,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.84</v>
+        <v>0.64</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1818,12 +1818,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Credit-to-GDP gap</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>credit_gap</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.186</v>
+        <v>0.264</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1840,16 +1840,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.49</v>
+        <v>-0.57</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1861,12 +1861,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private credit (% GDP)</t>
+          <t>Nominal GDP (log)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FS.AST.PRVT.GD.ZS</t>
+          <t>NGDPD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.179</v>
+        <v>0.235</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1887,17 +1887,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.157</v>
+        <v>0.217</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.47</v>
+        <v>0.62</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1947,12 +1947,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Net foreign assets growth</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nfa_g</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.147</v>
+        <v>0.202</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1969,11 +1969,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.32</v>
+        <v>-0.42</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.108</v>
+        <v>0.137</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.15</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2033,12 +2033,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Current account (% GDP)</t>
+          <t>Real effective exchange rate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BCA_NGDPD</t>
+          <t>BIS_REER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2047,15 +2047,15 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.103</v>
+        <v>0.126</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-0.42</v>
+        <v>0.62</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2076,12 +2076,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Real effective exchange rate</t>
+          <t>Current account (% GDP)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BIS_REER</t>
+          <t>BCA_NGDPD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2090,41 +2090,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.09</v>
+        <v>0.099</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.64</v>
+        <v>-0.08</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2133,24 +2133,24 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.057</v>
+        <v>0.029</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.51</v>
+        <v>-0.63</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2162,12 +2162,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2176,41 +2176,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.044</v>
+        <v>0.023</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>-0.47</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2219,15 +2219,15 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.035</v>
+        <v>0.017</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-0.24</v>
+        <v>-0.62</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2236,24 +2236,24 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.032</v>
+        <v>0.017</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2270,16 +2270,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-0.29</v>
+        <v>0.08</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.027</v>
+        <v>0.016</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-0.06</v>
+        <v>-0.23</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2334,12 +2334,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Loans-to-deposits</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>r_loans_dep</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2348,41 +2348,41 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.026</v>
+        <v>0.014</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-0.32</v>
+        <v>-0.05</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Loans-to-deposits</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>r_loans_dep</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2391,41 +2391,41 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.017</v>
+        <v>0.014</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>-0.31</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Log off-balance-sheet items</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>l_obsi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2434,41 +2434,41 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>-0.36</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2477,29 +2477,29 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.06</v>
+        <v>-0.6</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.014</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2549,12 +2549,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2563,41 +2563,41 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.33</v>
+        <v>0.08</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Log off-balance-sheet items</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>l_obsi</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2606,41 +2606,41 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.014</v>
+        <v>0.007</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.41</v>
+        <v>-0.08</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2649,41 +2649,41 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.012</v>
+        <v>0.007</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.12</v>
+        <v>0.54</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2700,16 +2700,16 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-0.02</v>
+        <v>-0.38</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2721,12 +2721,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2743,16 +2743,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>-0.05</v>
+        <v>0.44</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2764,12 +2764,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2786,7 +2786,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2807,12 +2807,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2829,11 +2829,11 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">

</xml_diff>

<commit_message>
Attribution rerun (13a-d, 14, 15) for seed 27
Replaces the attribution outputs that were stale copies from the initial commit.
Run on 24-09-2026 with tools/run_pipeline.py --only 13a 13b 13c 13d 14 15;
log in thesis-ews-final/outputs/run_logs/seed_attribution_2409.log.
Bank-level SHAP values stay out of the repository (gitignored, licensed data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/appendix_direction.xlsx
+++ b/outputs/tables/appendix_direction.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.927</v>
+        <v>0.989</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.87</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.654</v>
+        <v>0.736</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.571</v>
+        <v>0.579</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.55</v>
+        <v>-0.49</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.328</v>
+        <v>0.384</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -618,33 +618,33 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Inflation (CPI)</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PCPIPCH</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -653,41 +653,41 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.277</v>
+        <v>0.282</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.35</v>
+        <v>-0.49</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Inflation (CPI)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>PCPIPCH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -696,24 +696,24 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.256</v>
+        <v>0.255</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-0.42</v>
+        <v>0.41</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.119</v>
+        <v>0.191</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -756,7 +756,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.101</v>
+        <v>0.14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.51</v>
+        <v>0.59</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.091</v>
+        <v>0.105</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -854,12 +854,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -868,29 +868,29 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.055</v>
+        <v>0.053</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.48</v>
+        <v>0.85</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
@@ -911,41 +911,41 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.043</v>
+        <v>0.049</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.45</v>
+        <v>-0.79</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -954,24 +954,24 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.028</v>
+        <v>0.041</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.72</v>
+        <v>-0.53</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -983,12 +983,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Log loans</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>l_loans</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -997,41 +997,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.023</v>
+        <v>0.039</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-0.35</v>
+        <v>-0.36</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1040,41 +1040,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.018</v>
+        <v>0.023</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.33</v>
+        <v>-0.09</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>5/6</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1083,41 +1083,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.017</v>
+        <v>0.021</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.15</v>
+        <v>0.53</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1126,41 +1126,41 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>-0.6</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1169,41 +1169,41 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.02</v>
+        <v>-0.48</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1220,11 +1220,11 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.24</v>
+        <v>0.13</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Log loans</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>l_loans</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1263,16 +1263,16 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1306,11 +1306,11 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1327,12 +1327,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1341,15 +1341,15 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.02</v>
+        <v>-0.57</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1358,24 +1358,24 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1392,16 +1392,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>-0.05</v>
+        <v>-0.21</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1413,12 +1413,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1435,16 +1435,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-0.08</v>
+        <v>0.16</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1456,12 +1456,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.14</v>
+        <v>0.13</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.792</v>
+        <v>0.726</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.556</v>
+        <v>0.606</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.87</v>
+        <v>0.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.492</v>
+        <v>0.502</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.53</v>
+        <v>-0.55</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1689,12 +1689,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Credit growth</t>
+          <t>Change in net foreign assets (% GDP)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>credit_g</t>
+          <t>nfa_gdp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.293</v>
+        <v>0.322</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-0.7</v>
+        <v>-0.52</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1732,12 +1732,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Credit-to-GDP gap</t>
+          <t>Credit growth</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>credit_gap</t>
+          <t>credit_g</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.272</v>
+        <v>0.291</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1754,11 +1754,11 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-0.64</v>
+        <v>-0.42</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1775,12 +1775,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nominal GDP (log)</t>
+          <t>Private credit (% GDP)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NGDPD</t>
+          <t>FS.AST.PRVT.GD.ZS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.19</v>
+        <v>0.263</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1797,16 +1797,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.84</v>
+        <v>0.62</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1818,12 +1818,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Nominal GDP (log)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>NGDPD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1832,15 +1832,15 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.186</v>
+        <v>0.261</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.49</v>
+        <v>0.77</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1861,12 +1861,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private credit (% GDP)</t>
+          <t>Credit-to-GDP gap</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FS.AST.PRVT.GD.ZS</t>
+          <t>credit_gap</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1875,15 +1875,15 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.179</v>
+        <v>0.227</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.75</v>
+        <v>-0.63</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1892,24 +1892,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Inflation (CPI)</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PCPIPCH</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1918,24 +1918,24 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.157</v>
+        <v>0.197</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.47</v>
+        <v>-0.48</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Net foreign assets growth</t>
+          <t>Inflation (CPI)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nfa_g</t>
+          <t>PCPIPCH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1961,15 +1961,15 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.147</v>
+        <v>0.173</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.32</v>
+        <v>0.53</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.108</v>
+        <v>0.137</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2012,16 +2012,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.13</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2033,12 +2033,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Current account (% GDP)</t>
+          <t>Real effective exchange rate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BCA_NGDPD</t>
+          <t>BIS_REER</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2047,15 +2047,15 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.103</v>
+        <v>0.123</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-0.42</v>
+        <v>0.6</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2076,12 +2076,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Real effective exchange rate</t>
+          <t>Current account (% GDP)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BIS_REER</t>
+          <t>BCA_NGDPD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2090,41 +2090,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.09</v>
+        <v>0.092</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.64</v>
+        <v>-0.18</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2133,41 +2133,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.057</v>
+        <v>0.029</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.51</v>
+        <v>-0.65</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2176,41 +2176,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.044</v>
+        <v>0.024</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>-0.47</v>
+        <v>0.57</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.035</v>
+        <v>0.018</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2248,12 +2248,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2262,15 +2262,15 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-0.29</v>
+        <v>-0.61</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2279,24 +2279,24 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.027</v>
+        <v>0.016</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2313,16 +2313,16 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-0.06</v>
+        <v>0.13</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2348,7 +2348,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.026</v>
+        <v>0.015</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-0.32</v>
+        <v>-0.46</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2365,24 +2365,24 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Impairment charges</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>cr_impchg</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.017</v>
+        <v>0.014</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2399,16 +2399,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2420,12 +2420,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Log off-balance-sheet items</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>l_obsi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2434,29 +2434,29 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>-0.36</v>
+        <v>0.51</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2485,16 +2485,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2506,12 +2506,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Impairment charges</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cr_impchg</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.014</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17</v>
+        <v>0.24</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2549,12 +2549,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2563,41 +2563,41 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.33</v>
+        <v>0.23</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Log off-balance-sheet items</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>l_obsi</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2606,19 +2606,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.41</v>
+        <v>-0.45</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2628,19 +2628,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.12</v>
+        <v>-0.38</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-0.02</v>
+        <v>0.21</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2721,12 +2721,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>-0.05</v>
+        <v>0.3</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2764,12 +2764,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2786,7 +2786,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.05</v>
+        <v>-0.09</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.26</v>
+        <v>0.39</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">

</xml_diff>

<commit_message>
Attribution rerun (13a-d, 14, 15) for seed 99
Replaces the attribution outputs that were stale copies from the initial commit.
Run on 24-09-2026 with tools/run_pipeline.py --only 13a 13b 13c 13d 14 15;
log in thesis-ews-final/outputs/run_logs/seed_attribution_2409.log.
Bank-level SHAP values stay out of the repository (gitignored, licensed data).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/appendix_direction.xlsx
+++ b/outputs/tables/appendix_direction.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.927</v>
+        <v>0.997</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.86</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.654</v>
+        <v>0.773</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.571</v>
+        <v>0.636</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.55</v>
+        <v>-0.47</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.328</v>
+        <v>0.404</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -618,21 +618,21 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -653,11 +653,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.277</v>
+        <v>0.285</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.256</v>
+        <v>0.281</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.119</v>
+        <v>0.183</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -747,11 +747,11 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.05</v>
+        <v>0.27</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.101</v>
+        <v>0.137</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.51</v>
+        <v>0.58</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.091</v>
+        <v>0.109</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -854,12 +854,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -872,11 +872,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.48</v>
+        <v>0.9</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.043</v>
+        <v>0.048</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.45</v>
+        <v>-0.63</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -928,24 +928,24 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Log loans</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>l_loans</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -954,41 +954,41 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.028</v>
+        <v>0.04</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.72</v>
+        <v>-0.66</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.023</v>
+        <v>0.036</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-0.35</v>
+        <v>-0.64</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1026,12 +1026,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1040,41 +1040,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.33</v>
+        <v>-0.43</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1083,41 +1083,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1134,16 +1134,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1155,12 +1155,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1212,15 +1212,15 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.24</v>
+        <v>0.47</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1229,24 +1229,24 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Log loans</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>l_loans</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1255,15 +1255,15 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.21</v>
+        <v>-0.57</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1272,24 +1272,24 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1306,16 +1306,16 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>-0.4</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1327,12 +1327,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.014</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1349,16 +1349,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.02</v>
+        <v>0.33</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1370,12 +1370,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1392,16 +1392,16 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>-0.05</v>
+        <v>-0.18</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1413,12 +1413,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.006</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1435,16 +1435,16 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>-0.08</v>
+        <v>0.03</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1456,12 +1456,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.14</v>
+        <v>0.12</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.792</v>
+        <v>0.669</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-0.85</v>
+        <v>-0.87</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.556</v>
+        <v>0.518</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.492</v>
+        <v>0.442</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.53</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.293</v>
+        <v>0.243</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-0.7</v>
+        <v>-0.41</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1732,12 +1732,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Credit-to-GDP gap</t>
+          <t>Nominal GDP (log)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>credit_gap</t>
+          <t>NGDPD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1746,24 +1746,24 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.272</v>
+        <v>0.222</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-0.64</v>
+        <v>0.68</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1775,12 +1775,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nominal GDP (log)</t>
+          <t>Change in net foreign assets (% GDP)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NGDPD</t>
+          <t>nfa_gdp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1789,24 +1789,24 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.19</v>
+        <v>0.222</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.84</v>
+        <v>-0.54</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1818,12 +1818,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FX reserves (log)</t>
+          <t>Private credit (% GDP)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RXF11FX_REVS</t>
+          <t>FS.AST.PRVT.GD.ZS</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1832,15 +1832,15 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.186</v>
+        <v>0.221</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.49</v>
+        <v>0.63</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1861,12 +1861,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private credit (% GDP)</t>
+          <t>Credit-to-GDP gap</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FS.AST.PRVT.GD.ZS</t>
+          <t>credit_gap</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1875,15 +1875,15 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.179</v>
+        <v>0.194</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.75</v>
+        <v>-0.52</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1892,24 +1892,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Inflation (CPI)</t>
+          <t>FX reserves (log)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PCPIPCH</t>
+          <t>RXF11FX_REVS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1918,24 +1918,24 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.157</v>
+        <v>0.174</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.47</v>
+        <v>-0.41</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Net foreign assets growth</t>
+          <t>Inflation (CPI)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nfa_g</t>
+          <t>PCPIPCH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1961,15 +1961,15 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.147</v>
+        <v>0.148</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>-0.32</v>
+        <v>0.64</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1990,12 +1990,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FX reserves growth</t>
+          <t>Real effective exchange rate</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fx_g</t>
+          <t>BIS_REER</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2004,41 +2004,41 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.108</v>
+        <v>0.105</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Sign consistent, shape reverses</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Current account (% GDP)</t>
+          <t>FX reserves growth</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BCA_NGDPD</t>
+          <t>fx_g</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2047,41 +2047,41 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.103</v>
+        <v>0.097</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>-0.42</v>
+        <v>0.1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Real effective exchange rate</t>
+          <t>Current account (% GDP)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BIS_REER</t>
+          <t>BCA_NGDPD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2090,41 +2090,41 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.09</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.64</v>
+        <v>-0.01</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Log total assets</t>
+          <t>Net interest margin</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>l_assets</t>
+          <t>p_nim</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2133,41 +2133,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.057</v>
+        <v>0.028</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Higher → higher risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.51</v>
+        <v>-0.68</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Return on equity</t>
+          <t>Log total assets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>p_roe</t>
+          <t>l_assets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2176,41 +2176,41 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.044</v>
+        <v>0.027</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>-0.47</v>
+        <v>0.83</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deposits-to-liabilities</t>
+          <t>Gross loans</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>r_dep_liab</t>
+          <t>x_loans_gross</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.035</v>
+        <v>0.023</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2227,16 +2227,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-0.24</v>
+        <v>-0.21</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2248,12 +2248,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Net interest margin</t>
+          <t>Return on equity</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>p_nim</t>
+          <t>p_roe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2262,15 +2262,15 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.032</v>
+        <v>0.017</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-0.29</v>
+        <v>-0.5</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2284,19 +2284,19 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gross loans</t>
+          <t>Deposits-to-liabilities</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>x_loans_gross</t>
+          <t>r_dep_liab</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.027</v>
+        <v>0.016</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-0.06</v>
+        <v>-0.15</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2348,15 +2348,15 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.026</v>
+        <v>0.014</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-0.32</v>
+        <v>-0.24</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2365,24 +2365,24 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sign consistent, shape reverses</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cost-to-income ratio</t>
+          <t>Log off-balance-sheet items</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>r_cti</t>
+          <t>l_obsi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2391,41 +2391,41 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.017</v>
+        <v>0.014</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → higher risk</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Impairment charges</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c_leverage</t>
+          <t>cr_impchg</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2442,16 +2442,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>-0.36</v>
+        <v>0.08</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2463,12 +2463,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Equity ratio</t>
+          <t>Return on assets</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c_eqratio</t>
+          <t>p_roa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2477,41 +2477,41 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Higher → lower risk</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.06</v>
+        <v>-0.58</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>No clear direction</t>
+          <t>Consistent</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Impairment charges</t>
+          <t>Equity ratio</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cr_impchg</t>
+          <t>c_eqratio</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17</v>
+        <v>-0.09</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2549,12 +2549,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Return on assets</t>
+          <t>Cost-to-income ratio</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>p_roa</t>
+          <t>r_cti</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2563,15 +2563,15 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.014</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Higher → lower risk</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>-0.33</v>
+        <v>0.25</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2580,24 +2580,24 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>0/5</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>No clear direction</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Log off-balance-sheet items</t>
+          <t>Customer deposits</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>l_obsi</t>
+          <t>x_dep</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2606,7 +2606,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.41</v>
+        <v>0.33</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2635,12 +2635,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Interbank liabilities</t>
+          <t>Loans-to-assets</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>x_ib_liab</t>
+          <t>r_loans_assets</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-0.12</v>
+        <v>-0.38</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2678,12 +2678,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Operating income</t>
+          <t>Net interest income</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>inc_op</t>
+          <t>inc_nii</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2692,7 +2692,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2700,16 +2700,16 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-0.02</v>
+        <v>0.16</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2721,12 +2721,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Net interest income</t>
+          <t>Interbank liabilities</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>inc_nii</t>
+          <t>x_ib_liab</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>-0.05</v>
+        <v>0.16</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2764,12 +2764,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Loans-to-assets</t>
+          <t>Operating income</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>r_loans_assets</t>
+          <t>inc_op</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2786,16 +2786,16 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2807,12 +2807,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Customer deposits</t>
+          <t>Leverage</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>x_dep</t>
+          <t>c_leverage</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2829,16 +2829,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.26</v>
+        <v>0.1</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">

</xml_diff>